<commit_message>
Verifica settimanale (parte 1/2): 71 duplicati marcati cross-file
Deduplica globale su tutti i file .xlsx in /output (nomi normalizzati +
domini sito_web, con guardia su provincia/area per evitare falsi positivi
su catene multi-filiale). Le occorrenze duplicate sono annotate nel campo
note con "[DUPLICATO — vedi anche: <file_canonico>]"; le righe canoniche
(file più vecchio) restano invariate. Nessuna riga o file cancellato.

Il doppio controllo WebSearch sulle righe DA VERIFICARE UMANAMENTE dei
file nuovi è in corso in background; seguirà un secondo commit con gli
upgrade di stato_verifica, l'aggiornamento di weekly_verify_state.json e
il log.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLAeHJBUm8eZJoqNiASFPU
</commit_message>
<xml_diff>
--- a/output/2026-09-14_20_Croazia_Virovitico-podravska_Cleaning.xlsx
+++ b/output/2026-09-14_20_Croazia_Virovitico-podravska_Cleaning.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Sede a Bjelovar, fuori dalla contea. Il sito aziendale si dichiara unico rappresentante specializzato per la contea di Bjelovar-Bilogora e area limitrofa (Virovitica, Slatina, Đurđevac); nessun punto vendita fisico confermato in Virovitičko-podravska.</t>
+          <t>Sede a Bjelovar, fuori dalla contea. Il sito aziendale si dichiara unico rappresentante specializzato per la contea di Bjelovar-Bilogora e area limitrofa (Virovitica, Slatina, Đurđevac); nessun punto vendita fisico confermato in Virovitičko-podravska. [DUPLICATO — vedi anche: 2026-09-13_02_Croazia_Varazdinska_ATEX_Equipment-Services.xlsx]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Sede a Zagabria, fuori dalla contea. Distributore nazionale leader di settore con vendita/spedizione su tutta la Croazia; nessuna filiale fisica confermata in Virovitičko-podravska.</t>
+          <t>Sede a Zagabria, fuori dalla contea. Distributore nazionale leader di settore con vendita/spedizione su tutta la Croazia; nessuna filiale fisica confermata in Virovitičko-podravska. [DUPLICATO — vedi anche: 2026-09-07_19_Croazia_Zagrebacka_Depolverazione_Trattamento_aria.xlsx]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">

</xml_diff>